<commit_message>
dados: atualiza RA.xlsx/SP.xlsx com export completo das 3 bases
RA.xlsx anterior so cobria UTGC; novo export traz UTGC/TIMS/UTGSUL
completos (658 RAs), permitindo cruzar 100% das SPs com a data de
abertura real (antes so 54/123 SPs conseguiam essa data).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/SP.xlsx
+++ b/dados/SP.xlsx
@@ -6331,6 +6331,241 @@
         <v/>
       </c>
     </row>
+    <row r="125" ht="12.75">
+      <c r="A125" s="2" t="str">
+        <v>RA-327/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Providenciar o planejamento e implantação nas rotinas de manutenção e conservação de áreas verdes neste local.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="126" ht="12.75">
+      <c r="A126" s="2" t="str">
+        <v>RA-329/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Providenciar os itens solicitados nesta OM até a data deste RA.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="127" ht="12.75">
+      <c r="A127" s="2" t="str">
+        <v>RA-331/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o envio das LV's mencionadas neste RA até a medição do contrato.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="128" ht="12.75">
+      <c r="A128" s="2" t="str">
+        <v>RA-332/2026-SP-2</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos planejamento e execução da atividade até a data informada nesta Solicitação de Providência.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="129" ht="12.75">
+      <c r="A129" s="2" t="str">
+        <v>RA-333/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atendido</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGSUL</v>
+      </c>
+      <c s="2" t="str">
+        <v>A Petrobras notifica a empresa Normatel sobre a ausência do profissional designado na função de "planejador" para atuação nas instalações TIMS e UTGSUL. Determina o prazo até 10/07/2026 para regularização sob pena de sanção contratual.</v>
+      </c>
+      <c s="2" t="str">
+        <v>10/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>05/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezado Sr. Nelson.Em atendimento  Solicitao de Providncia RA-333/2026/SP-1, encaminhamos em anexo a resposta formal da NORMATEL ENGENHARIA LTDA, contendo os esclarecimentos sobre a alocao do profissional Planejador das instalaes TIMS e UTGSUL, a fundamentao contratual aplicvel (Anexo 1E  Recursos e Anexo 1J  Critrio de Medio) e as providncias assumidas, dentre elas a formalizao do Plano de Otimizao de Recursos para prvia avaliao dessa Fiscalizao.Permanecemos  disposio para reunio de alinhamento e apresentao de evidncias complementares.Atenciosamente,NORMATEL ENGENHARIA LTDA  Contrato 4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>05/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Resposta_RA-333-2026_SP-1_Normatel_v2_1.pdf</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
dados: atualiza Produttivo, ServiceNow e SAMC (RA/SP) para apresentacao
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/SP.xlsx
+++ b/dados/SP.xlsx
@@ -1542,7 +1542,7 @@
         <v>RA-559/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1560,7 +1560,7 @@
         <v>26/09/2025</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>A CONTRATADA informa esta FISCALIZAO que enviou os documentos pendentes via plataforma BROA. Em anexo, comprovante de envio dos documentos.</v>
@@ -1581,7 +1581,7 @@
         <v>EPMJ</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="24" ht="12.75">
@@ -1871,7 +1871,7 @@
         <v>RA-780/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1889,7 +1889,7 @@
         <v>23/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Informamos que o processo de contratao para a funo de Inspetor de Qualidade foi concludo.O profissional iniciou suas atividades em 20/01/2026 e encontra-se apto a atender plenamente as unidades UTGSUL e TIMS, conforme estabelecido em contrato.</v>
@@ -1910,7 +1910,7 @@
         <v>AINU</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="31" ht="12.75">
@@ -2294,7 +2294,7 @@
         <v>RA-96/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2312,7 +2312,7 @@
         <v>04/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>A contratada informa a esta fiscalizao que o histograma, que apresenta a rotatividade de colaboradores no projeto, assim como, a relao de colaboradores ativos, esto em anexo.;</v>
@@ -2333,7 +2333,7 @@
         <v>G63T</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="40" ht="12.75">
@@ -4832,7 +4832,7 @@
         <v>RA-268/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4847,19 +4847,19 @@
         <v>13/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder da Equipe A no dia 13/05/2026, a Normatel informa que tomou cincia da ocorrncia e das providncias requeridas.Esclarecemos que, to logo identificada a ausncia do profissional, foi realizada a reposio imediata por bombeiro civil devidamente capacitado e com conhecimento da rotina operacional da unidade, garantindo o atendimento ao planto e a continuidade da prestao dos servios, de forma a minimizar qualquer impacto operacional.Com o objetivo de evitar a recorrncia de situaes semelhantes, foram reforados os procedimentos internos de acompanhamento do efetivo e de acionamento de substituies, assegurando maior agilidade na recomposio das equipes e o atendimento s exigncias contratuais previstas no item 7.9.18.2.A Normatel reafirma seu compromisso com a excelncia na prestao dos servios, sempre prezando pela qualidade, segurana, continuidade operacional e pelo cumprimento das obrigaes contratuais estabelecidas junto  Petrobras. Permanecemos empenhados na melhoria contnua de nossos processos e na adoo das medidas necessrias para prevenir novas ocorrncias.Colocamo-nos  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4868,7 +4868,7 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4879,7 +4879,7 @@
         <v>RA-269/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4894,19 +4894,19 @@
         <v>14/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder da Equipe C no dia 14/05/2026, a Normatel informa que tomou cincia da ocorrncia e das determinaes constantes no referido registro.Esclarecemos que, ao ser identificada a ausncia do profissional, foi providenciada de forma imediata a substituio por bombeiro civil devidamente capacitado e com conhecimento da rotina operacional da unidade, garantindo o atendimento ao planto e o restabelecimento do efetivo, de forma a assegurar a continuidade da prestao dos servios.Com o objetivo de evitar a recorrncia de situaes dessa natureza, a Normatel reforou junto s equipes operacional e administrativa os procedimentos de controle do efetivo e de acionamento de substituies, visando garantir o pleno atendimento s exigncias contratuais, em especial ao disposto no item 7.9.18.2 do contrato.A Normatel reafirma seu compromisso com a excelncia, a qualidade e a continuidade dos servios prestados, sempre buscando atender s exigncias contratuais da Petrobras e mantendo elevados padres de desempenho operacional. Permanecemos empenhados na melhoria contnua de nossos processos, adotando as medidas necessrias para prevenir novas ocorrncias.Permanecemos  disposio para quaisquer esclarecimentos que se fizerem necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4915,7 +4915,7 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4973,7 +4973,7 @@
         <v>RA-272/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4991,7 +4991,7 @@
         <v>26/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em ateno  notificao referente ao uso de aparelhos celulares particulares por colaboradores da Normatel para tratativas relacionadas ao Contrato n 4600682358, informamos que a empresa j est realizando as tratativas necessrias para atendimento ao requisito contratual constante no Anexo 4  Requisitos de Computao Pessoal, clusula 1, subitem 1.2.Como medida imediata, a Normatel orientou formalmente todos os colaboradores envolvidos no contrato a utilizarem exclusivamente os dispositivos mveis corporativos para quaisquer comunicaes e tratativas junto  fiscalizao da Petrobras, no sendo permitido o uso de aparelhos particulares para assuntos relacionados ao contrato.Adicionalmente, visando centralizar e padronizar a comunicao entre a Contratada e a Fiscalizao, informamos os seguintes contatos corporativos para atendimento das demandas operacionais:Coordenao UTG Sul e TIMS  Leandro dos Santos NoronhaTelefone: (27) 99879-2365Equipe Operacional UTG SulTelefone: (27) 99789-9952Equipe Operacional TIMSTelefone: (21) 97233-9908Ressaltamos que a Normatel permanece adotando as aes necessrias para assegurar o pleno atendimento s exigncias contratuais, reforando internamente as orientaes aos colaboradores quanto ao correto uso dos recursos corporativos disponibilizados para execuo das atividades do contrato.Permanecemos  disposio para quaisquer esclarecimentos adicionais.Atenciosamente,</v>
@@ -5012,7 +5012,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="97" ht="12.75">
@@ -5208,7 +5208,7 @@
         <v>RA-280/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5226,7 +5226,7 @@
         <v>22/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Prezados,Em complemento  resposta anteriormente encaminhada, informamos que as aes corretivas solicitadas foram integralmente implementadas.Os contentores/organizadores destinados  segregao dos materiais de limpeza, EPIs e produtos qumicos foram recebidos e j se encontram em utilizao pelas equipes nas instalaes da UTGSUL, garantindo o acondicionamento adequado e separado dos itens, conforme orientado.Dessa forma, consideramos a pendncia atendida, permanecendo as aes de acompanhamento e fiscalizao em campo para assegurar a manuteno da conformidade e prevenir recorrncias.Anexamos as evidncias fotogrficas da adequao realizada.Atenciosamente,</v>
@@ -5247,7 +5247,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="102" ht="12.75">
@@ -5443,7 +5443,7 @@
         <v>RA-286/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5458,19 +5458,19 @@
         <v>27/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder no dia 25/05/2026 e  falta de resposta ao RA 282/26, a Normatel informa que tomou cincia da ocorrncia e das sanes aplicadas, comprometendo-se a reforar os controles internos para evitar a repetio de situaes dessa natureza.Esclarecemos que, to logo identificada a ausncia do profissional, foi providenciada de forma imediata a reposio do efetivo por profissional devidamente capacitado e com conhecimento da rotina operacional da unidade, garantindo a continuidade da prestao dos servios e evitando que o posto permanecesse desguarnecido durante o atendimento ao planto.Reconhecemos a importncia do cumprimento integral das obrigaes contratuais, especialmente no que se refere  manuteno ininterrupta do efetivo, conforme previsto no item 7.9.18.2 do contrato, motivo pelo qual reforamos junto  equipe operacional e de gesto os procedimentos de controle, comunicao e substituio de pessoal.A Normatel sempre pautou sua atuao pela qualidade, responsabilidade e excelncia na prestao dos servios, mantendo o compromisso com a segurana das operaes e com o atendimento s exigncias contratuais da Petrobras. Reiteramos nosso empenho em adotar todas as medidas necessrias para prevenir recorrncias e assegurar a continuidade dos servios com o padro de qualidade esperado.Permanecemos  disposio para quaisquer esclarecimentos adicionais.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5479,10 +5479,10 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="107" ht="12.75">
@@ -5537,7 +5537,7 @@
         <v>RA-288/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5552,19 +5552,19 @@
         <v>27/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder no dia 27/05/2026, a Normatel informa que tomou cincia da ocorrncia e das providncias decorrentes do registro.Esclarecemos que, ao ser identificada a ausncia do profissional, foi providenciada de imediato a reposio do efetivo por profissional devidamente capacitado e apto a desempenhar as atividades da funo, garantindo a continuidade da prestao dos servios e o atendimento ao planto, de forma a minimizar os impactos operacionais e restabelecer o efetivo no menor tempo possvel.Adicionalmente, informamos que foram reforados os procedimentos internos de controle e gesto do efetivo, com o objetivo de prevenir a recorrncia de situaes semelhantes e assegurar o pleno atendimento ao disposto no item 7.9.18.2 do contrato.A Normatel reafirma que sempre pautou sua atuao pela excelncia, qualidade e compromisso com a prestao dos servios, buscando atender s exigncias contratuais e s expectativas da Petrobras. Permanecemos empenhados na melhoria contnua de nossos processos e na adoo de todas as medidas necessrias para garantir a continuidade dos servios com segurana, eficincia e qualidade.Permanecemos  disposio para quaisquer esclarecimentos que se fizerem necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5573,10 +5573,10 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="109" ht="12.75">
@@ -5631,7 +5631,7 @@
         <v>RA-290/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5649,7 +5649,7 @@
         <v>03/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em atendimento  notificao emitida pela fiscalizao da Petrobras, informamos que a NORMATEL j realizou a reposio dos porta desodorizadores automticos nos ambientes das instalaes UTGSUL, atendendo ao disposto no ANEXO N 1 G  MATERIAIS, subitem 2.1.1.3 do Contrato n 4600682358.Seguem anexadas as evidncias da regularizao realizada.Dessa forma, consideramos a pendncia sanada, permanecendo  disposio para quaisquer esclarecimentos adicionais.</v>
@@ -5670,7 +5670,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="111" ht="12.75">
@@ -5678,7 +5678,7 @@
         <v>RA-297/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5693,19 +5693,19 @@
         <v>31/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder na instalao TIMS, no dia 31/05/2026, a Normatel informa que tomou cincia da ocorrncia e das determinaes constantes no referido registro.Esclarecemos que, to logo identificada a ausncia do profissional, foi realizada a reposio imediata do efetivo por bombeiro civil devidamente capacitado e com conhecimento das atividades operacionais da unidade, garantindo o atendimento ao planto e restabelecendo o posto de trabalho no menor tempo possvel, de modo a preservar a continuidade da prestao dos servios.Adicionalmente, foram reforados os procedimentos internos de controle e gesto do efetivo, com foco na pronta substituio de profissionais em casos de ausncias, visando assegurar o cumprimento integral das obrigaes contratuais estabelecidas no item 7.9.18.2.A Normatel reafirma seu compromisso com a excelncia na prestao dos servios, sempre prezando pela qualidade, segurana, continuidade operacional e atendimento s exigncias contratuais da Petrobras. Nesse sentido, permanecemos empenhados na adoo de medidas preventivas para evitar a recorrncia de situaes dessa natureza e garantir a manuteno dos padres de desempenho esperados.Permanecemos  disposio para quaisquer esclarecimentos adicionais.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5714,10 +5714,10 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="112" ht="12.75">
@@ -5725,7 +5725,7 @@
         <v>RA-298/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5743,7 +5743,7 @@
         <v>30/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em atendimento  notificao emitida pela fiscalizao, informamos que os servios solicitados foram devidamente executados.Foram realizadas a reinstalao e a reativao dos sensores de fumaa dos contineres (almoxarifado e escritrio), dos mdulos refeitrio e almoxarifado da brigada, localizados na lateral do galpo BASERV, bem como do escritrio da Segurana Patrimonial situado no galpo BASERV.Segue em anexo o registro fotogrfico evidenciando a execuo dos servios.Permanecemos  disposio para quaisquer esclarecimentos que se faam necessrios.Atenciosamente,</v>
@@ -5764,7 +5764,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="113" ht="12.75">
@@ -5866,7 +5866,7 @@
         <v>RA-306/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5881,28 +5881,28 @@
         <v>05/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento ao RA-306/2026, tendo em vista a extenso do contedo tcnico, encaminhamos em anexo a resposta completa referente aos itens SP-1 (Anlise de Falhas) e SP-2 (Plano de Ao com Medidas Corretivas e Preventivas).  Permanecemos  disposio para quaisquer esclarecimentos complementares que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Resposta_RA-306-2026_SP1_SP2.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5913,7 +5913,7 @@
         <v>RA-306/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5928,28 +5928,28 @@
         <v>05/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento ao RA-306/2026, tendo em vista a extenso do contedo tcnico, encaminhamos em anexo a resposta completa referente aos itens SP-1 (Anlise de Falhas) e SP-2 (Plano de Ao com Medidas Corretivas e Preventivas).Permanecemos  disposio para quaisquer esclarecimentos complementares que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>09/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Resposta_RA-306-2026_SP1_SP2.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6195,7 +6195,7 @@
         <v>RA-322/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6210,19 +6210,19 @@
         <v>30/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>10/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, a Normatel esclarece que sempre adotou todas as medidas necessrias para atender integralmente s exigncias contratuais, buscando profissional qualificado e que atendesse aos requisitos previstos para o cargo de Bombeiro Mestre.Diante da indisponibilidade de mo de obra local no Estado do Esprito Santo que atendesse aos critrios exigidos, foi contratada a colaboradora Geilda Maria de Sousa Silva (Identificador 73055311), profissional oriunda de outro estado, com o objetivo de garantir a continuidade dos servios e o cumprimento das obrigaes contratuais.Entretanto, em razo da divergncia de entendimento quanto  aceitao da referida profissional para a funo, e sempre visando atender s expectativas do cliente e manter a plena conformidade contratual, a colaboradora Geilda Maria de Sousa Silva foi desligada da funo.Informamos que o novo colaborador, Sr. Washigton Wilson, que ocupar o cargo de Bombeiro Mestre, j realizou o exame admissional e tem previso de incio das atividades em 15/07/2026.Reiteramos que a Normatel sempre atuou pautada pela boa-f, pelo cumprimento das obrigaes contratuais e pela busca das melhores solues para garantir a continuidade e a qualidade dos servios prestados. Entendemos que a situao decorreu de uma divergncia de interpretao quanto aos requisitos de aceitao do profissional anteriormente designado, no havendo, em nenhum momento, inteno de descumprir as disposies contratuais.Por fim, permanecemos  inteira disposio para quaisquer esclarecimentos adicionais e reafirmamos nosso compromisso em atender nosso cliente da melhor forma possvel, sempre prezando pela qualidade, segurana e excelncia na prestao dos servios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>10/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6231,7 +6231,7 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6427,19 +6427,19 @@
     </row>
     <row r="127" ht="12.75">
       <c r="A127" s="2" t="str">
-        <v>RA-331/2026-SP-1</v>
-      </c>
-      <c s="2" t="str">
-        <v>Em Atendimento</v>
-      </c>
-      <c s="2" t="str">
-        <v>4600682358</v>
-      </c>
-      <c s="2" t="str">
-        <v>UTGC</v>
-      </c>
-      <c s="2" t="str">
-        <v>Solicitamos o envio das LV's mencionadas neste RA até a medição do contrato.</v>
+        <v>RA-330/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o envio do planejamento da atividade até a data deste RA.</v>
       </c>
       <c s="2" t="str">
         <v>15/07/2026</v>
@@ -6474,19 +6474,19 @@
     </row>
     <row r="128" ht="12.75">
       <c r="A128" s="2" t="str">
-        <v>RA-332/2026-SP-2</v>
-      </c>
-      <c s="2" t="str">
-        <v>Em Atendimento</v>
-      </c>
-      <c s="2" t="str">
-        <v>4600682358</v>
-      </c>
-      <c s="2" t="str">
-        <v>UTGC</v>
-      </c>
-      <c s="2" t="str">
-        <v>Solicitamos planejamento e execução da atividade até a data informada nesta Solicitação de Providência.</v>
+        <v>RA-331/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o envio das LV's mencionadas neste RA até a medição do contrato.</v>
       </c>
       <c s="2" t="str">
         <v>15/07/2026</v>
@@ -6521,6 +6521,53 @@
     </row>
     <row r="129" ht="12.75">
       <c r="A129" s="2" t="str">
+        <v>RA-332/2026-SP-2</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos planejamento e execução da atividade até a data informada nesta Solicitação de Providência.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="130" ht="12.75">
+      <c r="A130" s="2" t="str">
         <v>RA-333/2026-SP-1</v>
       </c>
       <c s="2" t="str">
@@ -6561,6 +6608,288 @@
       </c>
       <c s="2" t="str">
         <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="131" ht="12.75">
+      <c r="A131" s="2" t="str">
+        <v>RA-336/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Cancelado</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o envio do planejamento da atividade até a data deste RA.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Cancelado</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="132" ht="12.75">
+      <c r="A132" s="2" t="str">
+        <v>RA-338/2026-SP-2</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o envio das evidências de realização da atividade até a data deste RA.</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="133" ht="12.75">
+      <c r="A133" s="2" t="str">
+        <v>RA-340/2026-SP-3</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Elaboração de um plano de ação com medidas corretivas e preventivas, de forma a evitar a reincidência do evento.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="134" ht="12.75">
+      <c r="A134" s="2" t="str">
+        <v>RA-340/2026-SP-4</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos a realização de análise de falhas para identificar as causas que levaram ao encerramento da OM no SAP sem a efetiva execução / conclusão do serviço.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="135" ht="12.75">
+      <c r="A135" s="2" t="str">
+        <v>RA-341/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos execução da instalação dos hidrômetros no local. REFORÇAMOS que desde DEZEMBRO/2025, esta fiscalização solicitou a devida instalação e até o momento sem previsão pela Contratada. Segue até a data, a informação de data para a devida Instalação destes equipamentos, onde permanece a penalização em DGI, até o efetivo e completo atendimento das OM's abertas para esta adequação.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="136" ht="12.75">
+      <c r="A136" s="2" t="str">
+        <v>RA-342/2026-SP-3</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em Atendimento</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o atendimento para fornecimento e utilização de água de REUSO na UTGC. Segue até a data, a informação para a devido fornecimento, onde permanece a penalização em DGI, até o efetivo e completo atendimento desta adequação.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
       </c>
       <c s="2" t="str">
         <v/>

</xml_diff>

<commit_message>
dados: atualiza RA.xlsx e SP.xlsx (SAMC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/SP.xlsx
+++ b/dados/SP.xlsx
@@ -649,7 +649,7 @@
         <v>RA-211/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -664,28 +664,28 @@
         <v>24/06/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento  RA-211/2025, informamos que seguem anexos os documentos referentes ao gerenciamento da gua para consumo humano na UTGC:Cronograma de higienizao dos reservatrios;Cronograma de anlise da qualidade da gua;Cronograma de manuteno e higienizao dos purificadores;Procedimento de higienizao dos purificadores.Os documentos foram atualizados conforme as rotinas operacionais previstas para a unidade. Diante do atendimento  solicitao, pedimos a anlise da fiscalizao e, estando a documentao em conformidade, o encerramento da presente RA.Solange OliveiraCoordenao de Meio Ambiente</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC -Cronograma Higienização de Reservatorio.png, Plano de monitoramento potabilidade UTGC - 2026.xlsx, Planilha de troca  elemento filtrante e limpeza de purificador.xlsx</v>
       </c>
       <c s="2" t="str">
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -696,7 +696,7 @@
         <v>RA-212/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -711,19 +711,19 @@
         <v>24/06/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento ao RA acima, informamos que foram tomadas medidas para sanar as alegaes citadas, bem como remanejamento de pessoal de limpeza para o atendimento conforme descrito. Informamos que aps anlise e remanejamento de pessoal estamos contratando, para inicio a partir do dia 22/09/2025, 02(dois) colaboradores para atendimento as demanda.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -732,7 +732,7 @@
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -743,7 +743,7 @@
         <v>RA-226/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -758,19 +758,19 @@
         <v>01/07/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Enviado via email</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -779,7 +779,7 @@
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -931,7 +931,7 @@
         <v>RA-264/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -946,28 +946,28 @@
         <v>04/07/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>06/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento ao item 01 do RA-264/2025, encaminhamos, em anexo, o Cronograma de Controle de Pragas e Vetores, contendo a programao das atividades previstas, incluindo as manutenes dos cintures interno e externo da unidade, conforme solicitado.Informamos que o cronograma contempla as periodicidades de execuo dos servios contratados, visando garantir o adequado planejamento e atendimento das atividades de controle de pragas e vetores na UTGC.Permanecemos  disposio para quaisquer esclarecimentos que se faam necessrios.Atenciosamente,Solange OliveiraNORMATEL; ENGENHARIA</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>06/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Cronograma_Controle_Pragas_2026_.xlsx</v>
       </c>
       <c s="2" t="str">
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1025,7 +1025,7 @@
         <v>RA-304/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1040,28 +1040,28 @@
         <v>11/07/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento ao RA-304/2025, informamos que foram adotadas as aes necessrias para regularizao dos itens apontados durante a vistoria realizada na ETA em 03/07/2025.O pHmetro destinado ao uso operacional foi disponibilizado  equipe, garantindo a continuidade do monitoramento e controle dos parmetros de qualidade da gua distribuda.Adicionalmente, foram reunidos e anexados os laudos de calibrao atualizados dos equipamentos de medio utilizados na unidade, incluindo o turbidmetro da ETE, conforme solicitado e em atendimento s exigncias normativas e boas prticas operacionais.Reforamos que a Normatel permanece acompanhando continuamente as condies operacionais da ETA e ETE, visando assegurar a confiabilidade dos processos e a conformidade contratual.At.te,Solange OliveiraNormatel Engenharia;Coordenao de Meio Ambiente</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>4680156-0-PT-sign.pdf, 4680158-0-PT-sign.pdf, 4680160-0-PT-sign.pdf, 26 601682 CERTIFICADOS MEDIDOR DE PH.pdf, 4680157-0-PT-sign.pdf, 4680159-0-PT-sign.pdf, 4680204-0-PT-sign.pdf</v>
       </c>
       <c s="2" t="str">
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1072,7 +1072,7 @@
         <v>RA-346/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1090,7 +1090,7 @@
         <v>29/07/2025</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Segue resposta a RA - 346Documentao anexa referente ao equipamento;PLATAFORMA ELTRICA SIGMA 16 (PEMT).E-mail com a documentao enviada em 21/07/2025 para Jeferson Clemente.</v>
@@ -1111,7 +1111,7 @@
         <v>AINU</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="14" ht="12.75">
@@ -1119,7 +1119,7 @@
         <v>RA-357/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1134,28 +1134,28 @@
         <v>23/07/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Bom diaA Normatel Engenharia informa que desde o questionamento dessa RA, vem tratando as inspees/limpeza e manuteno de canaletas atravs do Planejamento do SAP que desde ento vem sendo cumprido. Em anexo a essa solicitao de Providncia segue o planejamento e as OMs do SAP para essa atividade.AtcEduardo WallaceGerente de Projetos - UTGCNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Resumo do Plano de Limpeza de Canaletas - UTCG.pdf</v>
       </c>
       <c s="2" t="str">
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>F1QM</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1166,7 +1166,7 @@
         <v>RA-424/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1181,19 +1181,19 @@
         <v>15/08/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>As-built Quadro Eltrico K-24 - PL-822401 - Prazo: 26/07/2025 -Novo prazo: 03/10 para apresentao do projetoAtividade com maior complexidade e esta sendo alinhado junto ao sup. Ccero.06/10 - Disponibilizado ponto para mquina de caf na copa K-24.24/10 - Falta o projeto atualizado e assinado.06/11 - Atividade concludo</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1202,7 +1202,7 @@
         <v>DIDM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1213,7 +1213,7 @@
         <v>RA-471/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1228,19 +1228,19 @@
         <v>28/08/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Documentao enviada</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1249,7 +1249,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1260,7 +1260,7 @@
         <v>RA-479/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1275,19 +1275,19 @@
         <v>10/09/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Segue anexo as evidencias</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1296,7 +1296,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1307,7 +1307,7 @@
         <v>RA-491/2025-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1322,19 +1322,19 @@
         <v>08/09/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atividades vem sendo executadas conforme cronogramas sem falhas pontuais</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1343,7 +1343,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1354,7 +1354,7 @@
         <v>RA-503/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1369,28 +1369,28 @@
         <v>10/09/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,;Em atendimento  RA-503/2025, informamos que foram executadas as intervenes de manuteno na ETE da UTGC, incluindo a limpeza do reator UASB e a substituio dos elementos filtrantes (condutes) do filtro biolgico percolador.Encaminhamos, em anexo, o Relatrio de Manuteno da ETE, contendo a descrio dos servios realizados e os respectivos registros fotogrficos.Considerando a execuo e a documentao das atividades solicitadas, pedimos a anlise da fiscalizao e, estando o relatrio em conformidade, o encerramento da presente RA.Solange OliveiraCoordenao de Meio AmbienteNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>260302-Relatorio_ETE_UTGC_RevFinal_v00.pdf.crdownload</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1589,7 +1589,7 @@
         <v>RA-560/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1607,7 +1607,7 @@
         <v>26/09/2025</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>A CONTRATADA informa esta FISCALIZAO que enviou os documentos pendentes via plataforma BROA. Em anexo, comprovante de envio dos documentos.</v>
@@ -1628,7 +1628,7 @@
         <v>EPMJ</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="25" ht="12.75">
@@ -1777,7 +1777,7 @@
         <v>RA-725/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1792,28 +1792,28 @@
         <v>28/11/2025</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Foi realizada a recuperao dos corrimes das subestaes K-40, K-20, K-21, K-45 e K-38. Conforme solicitado, tambm foi efetuada a adequao dos aterramentos dos corrimes, garantindo a conformidade com os requisitos de segurana. Seguem, em anexo, fotos da atividade executada para registro e acompanhamento.Glaudstone CarvalhoSupervisor manuteno.Normatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-08-04 at 15.36.06.jpeg, WhatsApp Image 2026-08-04 at 15.36.07.jpeg, WhatsApp Image 2026-08-04 at 15.36.08 (1).jpeg, WhatsApp Image 2026-08-04 at 15.36.08.jpeg, WhatsApp Image 2026-08-04 at 15.36.08 (2).jpeg</v>
       </c>
       <c s="2" t="str">
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1824,7 +1824,7 @@
         <v>RA-764/2025-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1839,19 +1839,19 @@
         <v>09/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-764/2025, a CONTRATADA esclarece que est apurando internamente as circunstncias do encerramento das ordens 2030469144 e 2030469210 sem a execuo da substituio dos elementos filtrantes.Informamos que a atividade de substituio dos elementos filtrantes da ETA est sendo reprogramada, com reforo do controle de execuo antes do encerramento de ordens preventivas no SAP.Permanecemos  disposio para esclarecimentos adicionais.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1860,7 +1860,7 @@
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -1918,7 +1918,7 @@
         <v>RA-12/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1936,7 +1936,7 @@
         <v>23/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Segue Plano de Ao solicitado.</v>
@@ -1957,7 +1957,7 @@
         <v>AINU</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="32" ht="12.75">
@@ -1965,7 +1965,7 @@
         <v>RA-13/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -1980,28 +1980,28 @@
         <v>30/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>29/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>A Normatel Engenharia informa que foram implementadas as aes que contam no plano em anexo. Diante disso est finalizando a RA em questo.AtcEduardo WallaceGerente de ProjetoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v>29/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>AUDICOMP_descricao_desvios_UTGC.pdf, FG-SGI-019-01 - PLANO DE AÇÃO AUDICOMP 2025 - UTGC(FG-SGI-019).csv</v>
       </c>
       <c s="2" t="str">
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>F1QM</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2059,7 +2059,7 @@
         <v>RA-44/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2074,28 +2074,28 @@
         <v>23/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Conforme solicitado, foi realizada manuteno das placas de divisria da placas do auditrio, atividade foi acompanhada atividade pela fiscalizao e pelo tcnico de segurana Marlone, conforme evidenciado na foto em anexo.Atenciosamente,Glaudstone CarvalhoSupervisor de ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-08-04 at 09.35.57.jpeg</v>
       </c>
       <c s="2" t="str">
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2106,7 +2106,7 @@
         <v>RA-45/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2124,7 +2124,7 @@
         <v>23/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Seguem projetos atualizados.</v>
@@ -2145,7 +2145,7 @@
         <v>AINU</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="36" ht="12.75">
@@ -2153,7 +2153,7 @@
         <v>RA-51/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2168,19 +2168,19 @@
         <v>22/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>16/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em resposta ao RA Informativo, informamos que as atualizaes dos cards dos Planners no Microsoft Teams j esto sendo realizadas conforme a periodicidade estabelecida, buscando garantir que as informaes estejam disponveis antes das respectivas reunies.Ressaltamos, ainda, que o processo de gerenciamento e acompanhamento das atividades encontra-se em constante evoluo, com aes contnuas de aprimoramento voltadas ao fortalecimento dos controles,  melhoria da qualidade das informaes e ao atendimento das diretrizes contratuais estabelecidas pela Fiscalizao.Permanecemos  disposio para quaisquer esclarecimentos adicionais.</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMY7</v>
+      </c>
+      <c s="2" t="str">
+        <v>16/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2189,7 +2189,7 @@
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMY7</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2200,7 +2200,7 @@
         <v>RA-51/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2215,19 +2215,19 @@
         <v>26/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>16/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em resposta ao RA Informativo, informamos que as atualizaes dos cards dos Planners no Microsoft Teams j esto sendo realizadas conforme a periodicidade estabelecida, buscando garantir que as informaes estejam disponveis antes das respectivas reunies.Ressaltamos, ainda, que o processo de gerenciamento e acompanhamento das atividades encontra-se em constante evoluo, com aes contnuas de aprimoramento voltadas ao fortalecimento dos controles,  melhoria da qualidade das informaes e ao atendimento das diretrizes contratuais estabelecidas pela Fiscalizao.Permanecemos  disposio para quaisquer esclarecimentos adicionais.</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMY7</v>
+      </c>
+      <c s="2" t="str">
+        <v>16/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2236,7 +2236,7 @@
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMY7</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2247,7 +2247,7 @@
         <v>RA-51/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2262,19 +2262,19 @@
         <v>30/01/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>16/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em resposta ao RA Informativo, informamos que as atualizaes dos cards dos Planners no Microsoft Teams j esto sendo realizadas conforme a periodicidade estabelecida, buscando garantir que as informaes estejam disponveis antes das respectivas reunies.Ressaltamos, ainda, que o processo de gerenciamento e acompanhamento das atividades encontra-se em constante evoluo, com aes contnuas de aprimoramento voltadas ao fortalecimento dos controles,  melhoria da qualidade das informaes e ao atendimento das diretrizes contratuais estabelecidas pela Fiscalizao.Permanecemos  disposio para quaisquer esclarecimentos adicionais.</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMY7</v>
+      </c>
+      <c s="2" t="str">
+        <v>16/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2283,7 +2283,7 @@
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMY7</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2341,7 +2341,7 @@
         <v>RA-103/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2356,28 +2356,28 @@
         <v>04/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>06/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento ao RA-103/2026, informamos que a documentao solicitada foi levantada, atualizada e est sendo encaminhada em anexo para atendimento da solicitao.Esto sendo apresentados os seguintes documentos:FISPQ/FDS dos resduos de sade;Contrato/habilitao da empresa coletora e destinadora final dos RSS;Certificado de Destinao Final (CDF) referente aos MTRs informados;Notas Fiscais referentes s coletas dos MTRs citados;Lista de treinamento do POP aplicvel;Laudo de qualidade do ar-condicionado e da gua.Informamos ainda que os documentos passam a compor o acervo documental da unidade, permanecendo disponveis para consulta sempre que necessrio.Permanecemos  disposio para quaisquer esclarecimentos adicionais.Atenciosamente,Solange Oliveira;Normatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>06/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Licença de Transporte RSS - vence em 18.05.2027.pdf.crdownload, certificado_destinacao_final_163758.pdf.crdownload, certificado_destinacao_final_212972.pdf.crdownload, manifesto_2112936656.pdf.crdownload, manifesto_2113265083.pdf, manifesto_complementar_13308.pdf.crdownload, RelatorioRecManif_2112936656.pdf, Rotograma_de_residuos_UTGC_Normatel.pdf.crdownload, RelatorioRecManif_2113265083.pdf.crdownload</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2529,7 +2529,7 @@
         <v>RA-112/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2544,28 +2544,28 @@
         <v>24/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,;Em atendimento ao RA-102/2026, informamos que as aes solicitadas foram executadas, conforme evidncias apresentadas em anexo.Aps a concluso das atividades, foram restabelecidas as condies adequadas do local, atendendo ao solicitado no referido RA.Dessa forma, consideramos a demanda atendida e solicitamos, por gentileza, o encerramento do RA-102/2026.Atenciosamente,Solange OliveiraNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Relatorio_Encerramento_RA-112-2026_CATR-I_CANTEIRO NORMATEL.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2576,7 +2576,7 @@
         <v>RA-128/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2591,19 +2591,19 @@
         <v>11/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Foi dada melhoria no fluxo de entrega e tem funcionado</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2612,7 +2612,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2623,7 +2623,7 @@
         <v>RA-128/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2638,19 +2638,19 @@
         <v>11/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Nenhum fornecedor consta pendencias financeiras at a data de hoje.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2659,7 +2659,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2670,7 +2670,7 @@
         <v>RA-129/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2685,28 +2685,28 @@
         <v>15/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento  RA-129/2026, referente  indisponibilidade do sistema de produo e distribuio de gua de reso da UTGC, informamos que foram realizadas as aes operacionais necessrias para utilizao do sistema.Nos dias 11 e 12/08/2026, foi realizado acompanhamento operacional do processo de produo de gua de reso, contemplando as etapas de tratamento, retrolavagem dos filtros, filtrao, decantao, monitoramento de turbidez e transferncia da gua tratada.Durante a atividade, foram tratados 10 m de gua de reso, sendo posteriormente realizado o carregamento do caminho destinado ao transporte de gua no potvel e a utilizao da gua produzida na irrigao de rea verde da UTGC.Como evidncia do atendimento, segue anexo o Relatrio Tcnico de Acompanhamento Operacional do Tratamento, Filtrao e Utilizao de gua de Reso, contendo os registros das atividades executadas e as respectivas evidncias fotogrficas.Dessa forma, apresentamos as evidncias das aes realizadas em atendimento ao apontamento da RA-129/2026 e solicitamos a avaliao para encerramento do registro.Solange OliveiraNORMATEL ENGENHARIA</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Relatorio_Tecnico_Agua_Reuso_UTGC_11-12-08-2026_REV00.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2717,7 +2717,7 @@
         <v>RA-130/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2732,28 +2732,28 @@
         <v>14/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento ao RA-130/2026, referente  solicitao de documentao relacionada ao PGRSS e  atualizao da pasta de documentos legais do prdio K25  UTGC, encaminhamos, em anexo, a documentao pertinente para atendimento  solicitao da fiscalizao.Os documentos apresentados contemplam registros e evidncias relacionados  gesto, coleta, transporte, destinao e controle dos resduos de servios de sade, conforme aplicvel.Permanecemos  disposio para eventuais esclarecimentos e tratativas que se faam necessrias.Atenciosamente,Solange OliveiraNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>manifesto_2112936656.pdf.crdownload, manifesto_2113265083.pdf, Licença de Transporte RSS - vence em 18.05.2027.pdf.crdownload, Rotograma_de_residuos_UTGC_Normatel.pdf.crdownload, certificado_destinacao_final_163758.pdf.crdownload, certificado_destinacao_final_212972.pdf.crdownload, IT-LIM-003-740_REV1_PROCEDIMENTO_LIMPEZA_PREDIAL.docx</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2764,7 +2764,7 @@
         <v>RA-134/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2779,19 +2779,19 @@
         <v>24/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Desconsiderar</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2800,7 +2800,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2811,7 +2811,7 @@
         <v>RA-134/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2826,19 +2826,19 @@
         <v>18/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento  solicitao, informamos que a atividade foi devidamente concluda na unidade UTGC, com o registro fotogrfico do "antes" e "depois" da adequao dos locais, tendo sido a documentao encaminhada por e-mail  Fiscalizao  poca.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2847,7 +2847,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2858,7 +2858,7 @@
         <v>RA-138/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2873,19 +2873,19 @@
         <v>31/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao SP-1, a CONTRATADA informa que o plano de recuperao para saneamento das pendncias de compras est em elaborao, contemplando o cronograma de regularizao do fluxo de aquisio de materiais.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2894,7 +2894,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2905,7 +2905,7 @@
         <v>RA-138/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2920,19 +2920,19 @@
         <v>31/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao SP-2, a CONTRATADA informa que o fluxo interno de compras est sendo revisado, com identificao dos pontos de atraso desde a abertura da solicitao at a concluso do processo, para ajuste do planejamento e retomada da fluidez.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2941,7 +2941,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2952,7 +2952,7 @@
         <v>RA-138/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -2967,19 +2967,19 @@
         <v>31/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao SP-3, a CONTRATADA informa que est sendo estruturado o treinamento contnuo da equipe de compras, visando alinhar o processo aos padres esperados pela Petrobras.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2988,7 +2988,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -2999,7 +2999,7 @@
         <v>RA-138/2026-SP-4</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3014,19 +3014,19 @@
         <v>31/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao SP-4, a CONTRATADA informa que passar a apresentar relatrio gerencial quinzenal com a evoluo das compras, conforme solicitado.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3035,7 +3035,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3046,7 +3046,7 @@
         <v>RA-140/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3061,19 +3061,19 @@
         <v>23/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atividade j realizada</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3082,7 +3082,7 @@
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3140,7 +3140,7 @@
         <v>RA-144/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3155,19 +3155,19 @@
         <v>18/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Bom diaA Normatel informa que toda a questo de atrasos na medio da qualidade do AR foi resolvido e que os relatrios foram entregues a Petrobras, assim que finalizado. Abaixo segue o link com as pastas onde esto os documentos comprobatrios da execuo e resultados da qualidade do AR.;COMPARTILHADO/GIO/BCES/AOES - Documentos - REVISO DE LAUDOS DE QUALIDADE DE AR - Todos os DocumentosAtcEduardo WallaceGerente de Projeto - UTGC/UTGSUL/TIMSNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3176,7 +3176,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>F1QM</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3187,7 +3187,7 @@
         <v>RA-148/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3202,19 +3202,19 @@
         <v>26/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-148/2026/SP-1, a CONTRATADA informa que a reforma do banheiro do prdio K33 foi concluda.Colocamo-nos  disposio para vistoria de confirmao junto  Fiscalizao.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3223,7 +3223,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3234,7 +3234,7 @@
         <v>RA-149/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3249,28 +3249,28 @@
         <v>23/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Conforme solicitado, foi realizada a instalao do bebedouro industrial na rea do prdio K-33, piso inferior, conforme evidenciado na foto em anexo.Glaudstone CarvalhoSupervisor de ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-08-03 at 15.37.48.jpeg, WhatsApp Image 2026-08-03 at 15.37.49.jpeg</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3281,7 +3281,7 @@
         <v>RA-151/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3296,28 +3296,28 @@
         <v>27/03/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>11/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento ao RA-151/2026, informamos que foram realizadas as tratativas referentes aos coletores de resduos apontados durante as inspees de campo na UTGC.As aes contemplaram a substituio e adequao de coletores danificados ou sem tampa, regularizao das identificaes, reposio de recipientes e reorganizao dos pontos de coleta seletiva, conforme a necessidade verificada em cada local.Alm dos pontos mencionados no RA, foi realizado tambm um levantamento complementar em outros locais da unidade, com o objetivo de identificar e corrigir situaes semelhantes, promovendo maior padronizao e melhores condies para a correta segregao dos resduos.Encaminhamos, em anexo, o Relatrio de Execuo de Servio, contendo os registros fotogrficos das condies verificadas e das adequaes realizadas.Diante das aes executadas e das evidncias apresentadas, solicitamos o encerramento do RA-151/2026.Atenciosamente,Solange OlivreiraNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>11/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Relatorio_RA-151-2026_Coletores_Residuos.pdf.crdownload</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3375,7 +3375,7 @@
         <v>RA-167/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3390,28 +3390,28 @@
         <v>15/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, informamos que a Normatel atendeu integralmente ao cronograma estabelecido pela fiscalizao para a execuo das atividades relacionadas  desativao, desmobilizao e reativao dos sistemas de incndio no TIMS.As intervenes foram realizadas conforme o planejamento definido em conjunto com a fiscalizao, contemplando as etapas previstas para a desmobilizao e mobilizao dos mdulos habitacionais, de forma a garantir a continuidade da segurana dos locais e o restabelecimento das condies operacionais do Sistema de Deteco e Alarme de Incndio (SDAI) e dos demais componentes dos sistemas de incndio.Reiteramos que todas as atividades foram executadas em conformidade com as orientaes da fiscalizao e dentro do cronograma acordado, atendendo s demandas previstas para cada etapa do planejamento.A Normatel reafirma seu compromisso com a segurana, a qualidade dos servios prestados e o cumprimento das obrigaes contratuais, permanecendo  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-06-30 at 09.13.06 (3).jpeg, WhatsApp Image 2026-06-30 at 09.13.14.jpeg, WhatsApp Image 2026-06-30 at 09.14.18.jpeg</v>
       </c>
       <c s="2" t="str">
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3422,7 +3422,7 @@
         <v>RA-169/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3437,19 +3437,19 @@
         <v>30/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, informamos que a Normatel adotou as providncias necessrias para atendimento  solicitao da fiscalizao, realizando a regularizao do Alvar de Licena dos galpes junto ao CBMES, conforme requerido.Esclarecemos que a demanda foi atendida dentro do prazo previsto pela fiscalizao, em conformidade com as exigncias aplicveis.A Normatel reafirma seu compromisso com o cumprimento das obrigaes legais, regulatrias e contratuais, atuando de forma diligente para manter a regularidade de sua documentao e assegurar a conformidade de suas operaes.Permanecemos  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>14/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3458,10 +3458,10 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="64" ht="12.75">
@@ -3469,7 +3469,7 @@
         <v>RA-171/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3484,28 +3484,28 @@
         <v>30/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Os servios realizados por nossa empresa abrangem exclusivamente atividades de manuteno, as quais no exigem licenciamento ambiental, por no serem consideradas potencialmente poluidoras nem gerarem impacto ambiental significativo.Em funo disso, inclusive, a Vigilncia Sanitria, ao avaliar as atividades descritas em nosso CNPJ, concedeu a devida iseno, que segue em anexo.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>1. Declaração de Dispensa de Licenciamento Ambiental (1).pdf</v>
       </c>
       <c s="2" t="str">
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3516,7 +3516,7 @@
         <v>RA-172/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3531,28 +3531,28 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Conforme solicitado, seguem em anexo o PMOC e a ART</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>ART 0820260035274_PMOC- UTGC.assinada (1) (2).pdf, PMOC UTGC REV01 [assinado] (1).pdf</v>
       </c>
       <c s="2" t="str">
         <v>AJG8</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3563,7 +3563,7 @@
         <v>RA-175/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3578,19 +3578,19 @@
         <v>03/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>em atendimento  RA-175, informamos que os transformadores de utilizao foram retirados e que foi realizada a adequao de um rob para utilizao do equipamento, com o uso de tomadas steck.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3599,7 +3599,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3610,7 +3610,7 @@
         <v>RA-184/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3625,28 +3625,28 @@
         <v>03/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Informamos que foram realizados todos os testes hidrostticos (TH) das mangueiras de combate a incndio. Encaminhamos, em anexo, o relatrio contendo os resultados dos testes hidrostticos efetuados.Glaudstone Carvalho.Supervisor ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Laudo_008-001 - TH MANGUEIRAS.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3657,7 +3657,7 @@
         <v>RA-187/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3672,19 +3672,19 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Os procedimentos utilizado na estao se encontra na pasta do BDCO.Os tapetes isolantes j FORAM CALIBRADOS. Quanto s ferramentas, tambem foram calibrados.Foi realizado aquisio de 20 tapetes isolante 440V, aguardando chegada.;</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3693,7 +3693,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3704,7 +3704,7 @@
         <v>RA-188/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3719,28 +3719,28 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>11/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento ao RA-188/2026, informamos que a rotina de troca das roupas de cama e toalhas dos prdios K-27 e K-32 foi revisada, estabelecendo maior frequncia durante o perodo de utilizao das acomodaes, conforme a ocupao e a necessidade identificada.Tambm foi reforada junto  equipe a obrigatoriedade de inspeo de todo o material recebido aps a higienizao e antes de sua disponibilizao aos usurios. Os itens que apresentarem sujidade, danos, manchas ou qualquer condio inadequada sero imediatamente separados e encaminhados para nova higienizao ou substituio.As orientaes foram repassadas aos responsveis, e o atendimento permanecer sob acompanhamento, visando garantir a qualidade dos materiais fornecidos e o cumprimento dos requisitos contratuais aplicveis.Diante das aes implementadas, solicitamos o encerramento do RA-188/2026.Solange Oliveira / Ricardo PauloNORMATEL ENGENHARIA</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>11/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Relatorio_Acompanhamento_RA-188-2026_Ricardo_Paulo.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3751,7 +3751,7 @@
         <v>RA-189/2026-SP-4</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3766,28 +3766,28 @@
         <v>02/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,;Em atendimento ao RA-189/2026, informamos que foram realizadas as aes de manuteno dos dispositivos destinados ao controle de moscas, contemplando a limpeza/higienizao e a reposio do lquido atrativo.Como ao complementar, foi executado;Lista de Verificao (LV) para manuteno das armadilhas de pragas e vetores, visando padronizar a execuo e o registro das manutenes realizadas.As evidncias das aes executadas constam no relatrio anexo.Diante do atendimento das aes, solicitamos o encerramento do RA-189/2026.Atenciosamente,Solange OliveiraNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>LV_Manutenção_Armadilhas_Pragas e Vetores_K-26.pdf, Relatorio_Encerramento_RA-189-2026.pdf, POP_MANUTENCAO_ARMADILHAS_CAPTURA_INSETOS_VOADORES_Normatel_REV02.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3798,7 +3798,7 @@
         <v>RA-190/2026-SP-5</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3813,19 +3813,19 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>RA - respondido na epoca fora da SP. Atendido, cronogramas em execuo</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3834,7 +3834,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3845,7 +3845,7 @@
         <v>RA-191/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3863,7 +3863,7 @@
         <v>24/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Estamos providenciando a compra dos materiais:3 cilindros reserva (nmero de pedido 392),5 caixas de acondicionamento dos cilindros reservas (Nmero pedido 392,)Suporte para as APRs, equipamentos autnomos e suporte do extintor para veculo. Prazo; para o processo de compra at dia 17/05.</v>
@@ -3884,7 +3884,7 @@
         <v>G63T</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="73" ht="12.75">
@@ -3892,7 +3892,7 @@
         <v>RA-192/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3907,19 +3907,19 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Conforme informado  fiscalizao, as ordens foram baixadas de forma equivocada. Esclarecemos que elas foram lanadas na programao para levantamento de recursos e, por engano, foram baixadas como inspeo de campo.Informamos ainda que, conforme alinhado e planejado, as atividades de limpeza das elevatrias foram realizadas nos dias 11/04 e 12/04/2024, conforme acordado com a fiscalizao.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3928,7 +3928,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3939,7 +3939,7 @@
         <v>RA-193/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -3954,28 +3954,28 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>10/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento ao RA-193/2026, referente  manuteno e operao da Central de Armazenamento Temporrio de Resduos  CATR I, informamos que foram realizadas as seguintes adequaes:Os resduos de vidro foram segregados e acondicionados em recipiente exclusivo, devidamente identificado;As bacias plsticas utilizadas para o acondicionamento de resduos foram identificadas conforme o tipo e a classificao dos materiais;Foi implantada uma planilha para o controle da movimentao dos resduos na CATR I;Os resduos de madeira foram retirados do contato direto com o solo, acondicionados adequadamente e identificados;A caamba destinada aos resduos no reciclveis foi adequada  cor cinza e j se encontra em utilizao. Os resduos Classe I foram segregados e acondicionados em recipientes especficos, na cor laranja e devidamente identificados.A equipe responsvel tambm recebeu treinamento e orientaes sobre a correta segregao, identificao, acondicionamento e controle da movimentao dos resduos. Alm disso, foi reforada a rotina de inspeo e acompanhamento da CATR I, a fim de evitar a reincidncia das situaes apontadas.Como evidncias das aes realizadas, seguem anexos:Lista de presena do treinamento realizado;Planilha de Movimentao de Resduos;Planilha de Acompanhamento de Resduos;Planilha de Controle Anual de Resduos;Registro fotogrfico da caamba cinza destinada aos resduos no reciclveis, comprovando o atendimento da adequao solicitada.Diante das adequaes realizadas e das evidncias apresentadas, consideramos as pendncias sanadas.Solange Cndida de OliveiraNORMATEL ENGENHARIA</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>10/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Controle_de_residuos_UTCG_2026.xlsx, Treinamento preenchimento da planilha de movimentação de residuo.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -3986,7 +3986,7 @@
         <v>RA-194/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4001,31 +4001,31 @@
         <v>08/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, encaminhamos, em anexo, o PMOC (Plano de Manuteno, Operao e Controle) da UTG-Sul, devidamente atualizado, para atendimento  solicitao da fiscalizao.Esclarecemos que o documento encaminhado contempla as informaes vigentes referentes ao PMOC da unidade, em conformidade com os requisitos aplicveis.Permanecemos  disposio para prestar quaisquer esclarecimentos adicionais que se faam necessrios e reiteramos nosso compromisso com o atendimento s exigncias legais, regulatrias e contratuais, sempre buscando assegurar a qualidade e a conformidade dos servios prestados.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>PMOC UTGSUL 2026 assinado.pdf</v>
       </c>
       <c s="2" t="str">
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="76" ht="12.75">
@@ -4033,7 +4033,7 @@
         <v>RA-195/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4048,31 +4048,31 @@
         <v>06/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, informamos que a Normatel atendeu  solicitao da fiscalizao dentro do prazo estabelecido.Encaminhamos, em anexo, a relao completa e atualizada dos colaboradores alocados no TIMS, contendo as informaes de nome completo, nmero do identificador e funo desempenhada, em conformidade com o previsto contratualmente no Anexo 1E.Esclarecemos, ainda, que esta relao vem sendo encaminhada mensalmente, juntamente com as medies, conforme fluxo estabelecido, permanecendo a Normatel comprometida com a continuidade desse procedimento para atendimento aos requisitos de controle, conformidade e validao contratual.A Normatel reafirma seu compromisso com o cumprimento das obrigaes contratuais e permanece  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Efetivo 745.xlsx</v>
       </c>
       <c s="2" t="str">
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="77" ht="12.75">
@@ -4080,7 +4080,7 @@
         <v>RA-196/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4095,19 +4095,19 @@
         <v>06/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>A contratada informa a esta fiscalizao que est em anexo a lista contendo o nome dos colaboradores, cdigo identificador Petrobras e a funo desempenhada.;</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4116,7 +4116,7 @@
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4127,7 +4127,7 @@
         <v>RA-197/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4142,31 +4142,31 @@
         <v>06/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, informamos que a Normatel atendeu  solicitao da fiscalizao dentro do prazo estabelecido.Encaminhamos, em anexo, a relao completa e atualizada dos colaboradores alocados na UTG-Sul, contendo as informaes de nome completo, nmero do identificador e funo desempenhada, em conformidade com o previsto contratualmente no Anexo 1E.Esclarecemos, ainda, que esta relao vem sendo encaminhada mensalmente, juntamente com as medies, conforme fluxo estabelecido, permanecendo a Normatel comprometida com a continuidade desse procedimento para atendimento aos requisitos de controle, conformidade e validao contratual.A Normatel reafirma seu compromisso com o cumprimento das obrigaes contratuais e permanece  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>EFETIVO 739.xlsx</v>
       </c>
       <c s="2" t="str">
         <v>CMOL</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="79" ht="12.75">
@@ -4174,7 +4174,7 @@
         <v>RA-202/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4189,31 +4189,31 @@
         <v>16/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado sem Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno  notificao recebida, informamos que todas as orientaes apontadas pela fiscalizao foram devidamente atendidas.Conforme solicitado, foi realizada a substituio dos talabartes dos cintos de segurana, em atendimento s recomendaes apresentadas durante a inspeo gerencial realizada na UTGSUL.Encaminhamos, em anexo, as evidncias fotogrficas que comprovam a implementao das adequaes realizadas.A Normatel refora seu compromisso com a segurana, a sade e o meio ambiente (SMS), atuando de forma preventiva e corretiva para garantir a conformidade dos processos, a mitigao de riscos e a melhoria contnua de suas atividades.Permanecemos  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
+      </c>
+      <c s="2" t="str">
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>14/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-07-13 at 14.34.40.jpeg</v>
       </c>
       <c s="2" t="str">
         <v>PDKM</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>E5BE</v>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
       </c>
     </row>
     <row r="80" ht="12.75">
@@ -4221,7 +4221,7 @@
         <v>RA-203/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4236,28 +4236,28 @@
         <v>16/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>A CONTRATADA informa que segue em anexo o registro das tratativas realizadas. Ressaltamos que as atividades pendentes sero tratadas at dia 30/05/2026 conforme ordens de manuteno.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>RELATORIO INSPEC¿A¿O GERENCIAL - UTGC.pdf</v>
       </c>
       <c s="2" t="str">
         <v>PDKM</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4268,7 +4268,7 @@
         <v>RA-204/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4283,19 +4283,19 @@
         <v>08/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-204/2026, a CONTRATADA informa que j foram retomadas as rotinas dirias de limpeza nos prdios K33, K45, K55, K32 e K18, com regularizao dos checklists ausentes no K33, K26 e nos contineres E e F.Reforamos junto  equipe de superviso o acompanhamento dirio da frequncia e da qualidade de execuo, especialmente no prdio K33, para evitar reincidncia.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4304,7 +4304,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4315,7 +4315,7 @@
         <v>RA-217/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4330,19 +4330,19 @@
         <v>17/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-217/2026/SP-1, a CONTRATADA informa que a reposio dos kits de higiene pessoal e a implantao dos dispensadores nos prdios K27 e K32 esto sendo regularizadas, e as evidncias de realizao sero encaminhadas  Fiscalizao.Reforamos o alinhamento com a equipe de hotelaria para o envio mensal dos itens 7.9.15.14 e 7.9.15.15 junto  medio, conforme previsto.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4351,7 +4351,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4362,7 +4362,7 @@
         <v>RA-236/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4377,28 +4377,28 @@
         <v>28/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Informamos que as evidncias da habilitao da equipe para atendimento a rea da sade foram enviadas via e-mail, conforme anexo.;</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>e-mail treinamento área da saúde.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4409,7 +4409,7 @@
         <v>RA-241/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4424,19 +4424,19 @@
         <v>10/04/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-241/2026/SP-1, a CONTRATADA informa que a rotina de troca de roupas de cama e toalhas foi ajustada para maior frequncia durante a estadia dos ocupantes nos prdios K27 e K32, alm da inspeo do material fornecido para substituio dos itens com desgaste.O envio semanal das evidncias dessas trocas ser providenciado  Fiscalizao.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4445,7 +4445,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4456,7 +4456,7 @@
         <v>RA-242/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4471,19 +4471,19 @@
         <v>07/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao SP-2, a CONTRATADA informa que est sendo providenciado o treinamento/reforo em DSMS junto aos profissionais da empresa responsvel pela movimentao de roupas de cama/banho, uniformes e EPIs, quanto aos requisitos de SMS relativos a acesso, permanncia e estacionamento nas instalaes.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4492,7 +4492,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4503,7 +4503,7 @@
         <v>RA-242/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4518,19 +4518,19 @@
         <v>07/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao SP-3, a CONTRATADA informa que o treinamento/reforo quanto ao armazenamento e movimentao adequados desses materiais, em conformidade com a legislao e os itens de SMS do Contrato, est sendo programado junto  empresa responsvel, com envio posterior da evidncia  Fiscalizao.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4539,7 +4539,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4550,7 +4550,7 @@
         <v>RA-247/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4565,19 +4565,19 @@
         <v>11/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados, reconhecemos o apontamento e a reincidncia registrada neste RA. Assumimos o compromisso de regularizar em definitivo o item, com acompanhamento direto da nossa coordenao.; informamos as providncias adotadas quanto ao ponto apontado pela Fiscalizao, com a regularizao em andamento.;</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4586,7 +4586,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4644,7 +4644,7 @@
         <v>RA-249/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4659,19 +4659,19 @@
         <v>04/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>A Contratada informa que, todas os equipamentos so a bateria.;Ainda temos alguns que utilizamos para aumento da produtividade, porem a fiscalizao local est ciente.;</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4680,7 +4680,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4691,7 +4691,7 @@
         <v>RA-250/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4706,19 +4706,19 @@
         <v>12/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Ser realizado por OBRAS</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4727,7 +4727,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4738,7 +4738,7 @@
         <v>RA-253/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4753,19 +4753,19 @@
         <v>16/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>RA respondido no numero;325/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4774,7 +4774,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4785,7 +4785,7 @@
         <v>RA-267/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4800,28 +4800,28 @@
         <v>29/05/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>03/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento  solicitao, foi realizada a substituio das placas de forro danificadas, bem como a fixao dos componentes necessrios para garantir a estabilidade e a segurana da instalao.Seguem anexas as evidncias fotogrficas da execuo do servio e das condies finais do local aps a interveno.Glaudstone Carvalho.Supervisor de ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>03/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-08-03 at 13.05.53.jpeg</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -4832,7 +4832,7 @@
         <v>RA-268/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4850,7 +4850,7 @@
         <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder da Equipe A no dia 13/05/2026, a Normatel informa que tomou cincia da ocorrncia e das providncias requeridas.Esclarecemos que, to logo identificada a ausncia do profissional, foi realizada a reposio imediata por bombeiro civil devidamente capacitado e com conhecimento da rotina operacional da unidade, garantindo o atendimento ao planto e a continuidade da prestao dos servios, de forma a minimizar qualquer impacto operacional.Com o objetivo de evitar a recorrncia de situaes semelhantes, foram reforados os procedimentos internos de acompanhamento do efetivo e de acionamento de substituies, assegurando maior agilidade na recomposio das equipes e o atendimento s exigncias contratuais previstas no item 7.9.18.2.A Normatel reafirma seu compromisso com a excelncia na prestao dos servios, sempre prezando pela qualidade, segurana, continuidade operacional e pelo cumprimento das obrigaes contratuais estabelecidas junto  Petrobras. Permanecemos empenhados na melhoria contnua de nossos processos e na adoo das medidas necessrias para prevenir novas ocorrncias.Colocamo-nos  disposio para quaisquer esclarecimentos adicionais que se faam necessrios.</v>
@@ -4871,7 +4871,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="94" ht="12.75">
@@ -4879,7 +4879,7 @@
         <v>RA-269/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4897,7 +4897,7 @@
         <v>09/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em ateno  notificao emitida por essa Fiscalizao, referente  ausncia do Bombeiro Civil Lder da Equipe C no dia 14/05/2026, a Normatel informa que tomou cincia da ocorrncia e das determinaes constantes no referido registro.Esclarecemos que, ao ser identificada a ausncia do profissional, foi providenciada de forma imediata a substituio por bombeiro civil devidamente capacitado e com conhecimento da rotina operacional da unidade, garantindo o atendimento ao planto e o restabelecimento do efetivo, de forma a assegurar a continuidade da prestao dos servios.Com o objetivo de evitar a recorrncia de situaes dessa natureza, a Normatel reforou junto s equipes operacional e administrativa os procedimentos de controle do efetivo e de acionamento de substituies, visando garantir o pleno atendimento s exigncias contratuais, em especial ao disposto no item 7.9.18.2 do contrato.A Normatel reafirma seu compromisso com a excelncia, a qualidade e a continuidade dos servios prestados, sempre buscando atender s exigncias contratuais da Petrobras e mantendo elevados padres de desempenho operacional. Permanecemos empenhados na melhoria contnua de nossos processos, adotando as medidas necessrias para prevenir novas ocorrncias.Permanecemos  disposio para quaisquer esclarecimentos que se fizerem necessrios.</v>
@@ -4918,7 +4918,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="95" ht="12.75">
@@ -4926,7 +4926,7 @@
         <v>RA-271/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -4944,7 +4944,7 @@
         <v>26/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em ateno  notificao referente ao uso de aparelhos celulares particulares por colaboradores da Normatel para tratativas relacionadas ao Contrato n 4600682358, informamos que a empresa j est realizando as tratativas necessrias para atendimento ao requisito contratual constante no Anexo 4  Requisitos de Computao Pessoal, clusula 1, subitem 1.2.Como medida imediata, a Normatel orientou formalmente todos os colaboradores envolvidos no contrato a utilizarem exclusivamente os dispositivos mveis corporativos para quaisquer comunicaes e tratativas junto  fiscalizao da Petrobras, no sendo permitido o uso de aparelhos particulares para assuntos relacionados ao contrato.Adicionalmente, visando centralizar e padronizar a comunicao entre a Contratada e a Fiscalizao, informamos os seguintes contatos corporativos para atendimento das demandas operacionais:Coordenao UTG Sul e TIMS  Leandro dos Santos NoronhaTelefone: (27) 99879-2365Equipe Operacional UTG SulTelefone: (27) 99789-9952Equipe Operacional TIMSTelefone: (21) 97233-9908Ressaltamos que a Normatel permanece adotando as aes necessrias para assegurar o pleno atendimento s exigncias contratuais, reforando internamente as orientaes aos colaboradores quanto ao correto uso dos recursos corporativos disponibilizados para execuo das atividades do contrato.Permanecemos  disposio para quaisquer esclarecimentos adicionais.Atenciosamente,</v>
@@ -4965,7 +4965,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="96" ht="12.75">
@@ -5302,7 +5302,7 @@
         <v>RA-283/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5317,19 +5317,19 @@
         <v>15/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>RA respondido no;325/2026, o mesmo cita esse RA e mais 2.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5338,7 +5338,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5349,7 +5349,7 @@
         <v>RA-284/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5364,19 +5364,19 @@
         <v>15/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>RA respondido no;325/2026, o mesmo cita este RA e mais 2. Os anexos atendem a ampla resposta</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5385,7 +5385,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5396,7 +5396,7 @@
         <v>RA-285/2026-SP-4</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5411,19 +5411,19 @@
         <v>15/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno ao RA-285/2026 referente  ausncia de profissional previsto no contrato, esclarecemos que o mesmo est no contrato a 2 meses.; (UESLEI)</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5432,7 +5432,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5772,7 +5772,7 @@
         <v>RA-304/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5787,19 +5787,19 @@
         <v>08/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados, reconhecemos o apontamento e a reincidncia registrada neste RA. Assumimos o compromisso de regularizar em definitivo o item, com acompanhamento direto da nossa coordenao.; informamos as providncias adotadas para normalizar o sistema de gua de reuso da UTGC. Estamos executando as intervenes necessrias e apresentamos o cronograma de concluso, com as medidas de contingncia aplicadas enquanto a normalizao no se conclui.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5808,7 +5808,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5819,7 +5819,7 @@
         <v>RA-305/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5834,28 +5834,28 @@
         <v>08/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento  RA-305/2026, referente  indisponibilidade do sistema de produo e distribuio de gua de reso da UTGC, informamos que foram realizadas as aes operacionais necessrias para utilizao do sistema.Nos dias 11 e 12/08/2026, foi realizado acompanhamento operacional do processo de produo de gua de reso, contemplando as etapas de tratamento, retrolavagem dos filtros, filtrao, decantao, monitoramento de turbidez e transferncia da gua tratada.Durante a atividade, foram tratados 10 m de gua de reso, sendo posteriormente realizado o carregamento do caminho destinado ao transporte de gua no potvel e a utilizao da gua produzida na irrigao de rea verde da UTGC.Como evidncia do atendimento, segue anexo o Relatrio Tcnico de Acompanhamento Operacional do Tratamento, Filtrao e Utilizao de gua de Reso, contendo os registros das atividades executadas e as respectivas evidncias fotogrficas.Dessa forma, apresentamos as evidncias das aes realizadas em atendimento ao apontamento da RA-305/2026 e solicitamos a avaliao para encerramento do registro.Solange OliveiraNORMATEL ENGENHARIA</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Relatorio_Tecnico_Agua_Reuso_UTGC_11-12-08-2026_REV00.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -5960,7 +5960,7 @@
         <v>RA-307/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -5975,28 +5975,28 @@
         <v>05/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>03/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Foi realizada a coleta em 24/04/2026, com emisso dos resultados em 04/05/2026, conforme apresentado no relatrio anexo.Aps a anlise dos parmetros identificados, foram avaliadas as no conformidades apontadas e propostas aes corretivas para tratamento das anomalias verificadas, de acordo com o relatrio de inspeo anexo.As aes propostas sero implementadas e uma nova coleta est programada para 28/08/2026, com o objetivo de verificar a eficcia das medidas adotadas.Glaudstone CarvalhoSupervisor de manutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>03/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>LAUDOS UTGCC qualidade de ar.pdf, Plano de ação analise de Ar RV.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6007,7 +6007,7 @@
         <v>RA-308/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6022,28 +6022,28 @@
         <v>16/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em atendimento ao RA-308/2026, informamos que foi realizada a reviso do procedimento de limpeza e conservao dos banheiros da UTGC, contemplando a incluso do controle para substituio mensal das telas/placas perfumadas dos mictrios, conforme solicitado.Adicionalmente, foi implantado o checklist de controle dos banheiros, permitindo o registro e acompanhamento sistemtico das atividades executadas, incluindo a verificao das condies de limpeza e dos itens previstos no procedimento.Com essas aes, a rotina passa a contar com controle formal para acompanhamento das atividades e atendimento ao estabelecido no Plano Bsico de Conservao e Limpeza.Diante das providncias adotadas, solicitamos a gentileza de considerar o RA-308/2026 atendido e proceder com o seu encerramento.Solange OliveiraNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>07/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>IT-LIM-005-740_Procedimento_Limpeza_Banheiros_Vestiarios_R1.pdf, Check list de banheiros.xlsx</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>GK42</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6054,7 +6054,7 @@
         <v>RA-311/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6069,19 +6069,19 @@
         <v>19/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Em ateno ao RA-311/2026/SP-2, a CONTRATADA informa que o levantamento das informaes solicitadas  estrutura operacional por setor, organograma, ambientes atendidos, atividades e periodicidades, alm do dimensionamento e distribuio da mo de obra  est sendo consolidado para envio via RA/e-mail  Fiscalizao.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6090,7 +6090,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6101,7 +6101,7 @@
         <v>RA-312/2026-SP-6</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6116,28 +6116,28 @@
         <v>16/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Segue cronograma em anexo</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>CRONOGRAMA DE POSTES.xlsx</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6148,7 +6148,7 @@
         <v>RA-317/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6163,28 +6163,28 @@
         <v>24/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Foram realizados. em anexo os relatrios</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>206733-2026 - 1-0.pdf, 206739-2026 - 1-0.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6195,7 +6195,7 @@
         <v>RA-322/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6213,7 +6213,7 @@
         <v>10/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Em ateno  notificao recebida, a Normatel esclarece que sempre adotou todas as medidas necessrias para atender integralmente s exigncias contratuais, buscando profissional qualificado e que atendesse aos requisitos previstos para o cargo de Bombeiro Mestre.Diante da indisponibilidade de mo de obra local no Estado do Esprito Santo que atendesse aos critrios exigidos, foi contratada a colaboradora Geilda Maria de Sousa Silva (Identificador 73055311), profissional oriunda de outro estado, com o objetivo de garantir a continuidade dos servios e o cumprimento das obrigaes contratuais.Entretanto, em razo da divergncia de entendimento quanto  aceitao da referida profissional para a funo, e sempre visando atender s expectativas do cliente e manter a plena conformidade contratual, a colaboradora Geilda Maria de Sousa Silva foi desligada da funo.Informamos que o novo colaborador, Sr. Washigton Wilson, que ocupar o cargo de Bombeiro Mestre, j realizou o exame admissional e tem previso de incio das atividades em 15/07/2026.Reiteramos que a Normatel sempre atuou pautada pela boa-f, pelo cumprimento das obrigaes contratuais e pela busca das melhores solues para garantir a continuidade e a qualidade dos servios prestados. Entendemos que a situao decorreu de uma divergncia de interpretao quanto aos requisitos de aceitao do profissional anteriormente designado, no havendo, em nenhum momento, inteno de descumprir as disposies contratuais.Por fim, permanecemos  inteira disposio para quaisquer esclarecimentos adicionais e reafirmamos nosso compromisso em atender nosso cliente da melhor forma possvel, sempre prezando pela qualidade, segurana e excelncia na prestao dos servios.</v>
@@ -6234,7 +6234,7 @@
         <v>E5BE</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="123" ht="12.75">
@@ -6242,7 +6242,7 @@
         <v>RA-325/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6257,28 +6257,28 @@
         <v>15/06/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Segue evidencias;</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>NOTA FISCAL CILINDROS CO2  17-07-26.pdf, INSPEÇÕES - EXTINTORES (1).pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6289,7 +6289,7 @@
         <v>RA-326/2026-SP-3</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6304,28 +6304,28 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Conforme solicitado, foi realizada a inspeo nos equipamentos, piso inferior, conforme evidenciado em anexo.Glaudstone CarvalhoSupervisor de ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>INSPEÇÕES - EXTINTORES (1).pdf, NOTA FISCAL CILINDROS CO2  17-07-26.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>RA-327/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6351,28 +6351,28 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>27/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>O Plano de reas Verdes j est implementado no SAP conforme anexo. As ordens so planejadas e impressas conforme as datas de execuo. A Normatel utiliza a programao do SAP para executar as atividades de Capinao,; Jardinagem e Servios de Poda.Segue em Anexo o Plano de Capinao da UTGC e o Ultimo relatrio dos Servios Realizados no Cinturo Verde.AtcEduardo; WallaceGerente de ProjetoNormatel EngenhariaChave: F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v>F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v>27/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>plano de area verde UTGC (1).xlsx, Relatório_Limpeza do Cinturão Verde.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>F1QM</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6383,7 +6383,7 @@
         <v>RA-329/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6398,28 +6398,28 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Foi realizada a instalao de algumas placas na rea das rotas operacionais, conforme demonstrado nas fotos em anexo. Tambm foi realizada a aquisio das placas que ainda estavam pendentes. A instalao desses itens est programada para ocorrer entre os dias 12/08 e 14/08.Glaudstone CarvalhoSupervisor de ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>04/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>WhatsApp Image 2026-08-04 at 10.07.01.jpeg, WhatsApp Image 2026-08-04 at 10.09.19.jpeg, WhatsApp Image 2026-08-04 at 10.10.44.jpeg</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6430,7 +6430,7 @@
         <v>RA-330/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6445,19 +6445,19 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-330/2026, a CONTRATADA informa que a atualizao da OM 2030719050 no PLANNER est sendo providenciada, e o planejamento da execuo da substituio dos postes de CFT na rea operacional est em elaborao junto  equipe de manuteno.Reforamos o acompanhamento da atividade para evitar novas postergaes, considerando o risco  segurana j apontado.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6466,7 +6466,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6477,7 +6477,7 @@
         <v>RA-331/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6492,28 +6492,28 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>03/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados, boa tarde.Glaudstone CarvalhoSupervisor de ManutenoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>03/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>ORDEM HIDROSSANITARIO.pdf, ORDEM HIDROSSANITARIO.pdf, Captura de tela 2026-08-03 154629.png</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6524,7 +6524,7 @@
         <v>RA-332/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6539,19 +6539,19 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-332/2026, a CONTRATADA informa que o planejamento para execuo do reparo do forro da escada de acesso ao auditrio est sendo priorizado, com a atividade sendo programada junto  equipe de manuteno para adequao imediata.Reforamos o esforo para regularizao do item, considerando a recorrncia j registrada desde 2025.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6571,7 +6571,7 @@
         <v>RA-333/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Atendido</v>
+        <v>Concluido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6589,7 +6589,7 @@
         <v>05/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v>Registrado com Pendência</v>
+        <v>Registrado sem Pendência</v>
       </c>
       <c s="2" t="str">
         <v>Prezado Sr. Nelson.Em atendimento  Solicitao de Providncia RA-333/2026/SP-1, encaminhamos em anexo a resposta formal da NORMATEL ENGENHARIA LTDA, contendo os esclarecimentos sobre a alocao do profissional Planejador das instalaes TIMS e UTGSUL, a fundamentao contratual aplicvel (Anexo 1E  Recursos e Anexo 1J  Critrio de Medio) e as providncias assumidas, dentre elas a formalizao do Plano de Otimizao de Recursos para prvia avaliao dessa Fiscalizao.Permanecemos  disposio para reunio de alinhamento e apresentao de evidncias complementares.Atenciosamente,NORMATEL ENGENHARIA LTDA  Contrato 4600682358</v>
@@ -6610,7 +6610,7 @@
         <v>DUHJ</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CMOL</v>
       </c>
     </row>
     <row r="131" ht="12.75">
@@ -6665,7 +6665,7 @@
         <v>RA-338/2026-SP-2</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6680,28 +6680,28 @@
         <v>31/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Conforme solicitado, foi realizada uma avaliao para a instalao de infraestrutura eltrica destinada  automatizao dos portes localizados na rea operacional do K-55, referente  OM 2031829575.A equipe realizou uma vistoria no local e identificou duas possveis alternativas para a alimentao eltrica dos portes da Rua 19 avaliao em anexo.</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Avaliação de infra k-55.pdf</v>
       </c>
       <c s="2" t="str">
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>CIEA</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6806,7 +6806,7 @@
         <v>RA-341/2026-SP-1</v>
       </c>
       <c s="2" t="str">
-        <v>Em Atendimento</v>
+        <v>Atendido</v>
       </c>
       <c s="2" t="str">
         <v>4600682358</v>
@@ -6821,19 +6821,19 @@
         <v>15/07/2026</v>
       </c>
       <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v>Registrado com Pendência</v>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
-      </c>
-      <c s="2" t="str">
-        <v/>
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados, reconhecemos o apontamento e a reincidncia registrada neste RA. Assumimos o compromisso de regularizar em definitivo o item, com acompanhamento direto da nossa coordenao.; informamos as providncias adotadas para normalizar o sistema de gua de reuso da UTGC. Estamos executando as intervenes necessrias e apresentamos o cronograma de concluso, com as medidas de contingncia aplicadas enquanto a normalizao no se conclui.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6842,7 +6842,7 @@
         <v>MP00</v>
       </c>
       <c s="2" t="str">
-        <v/>
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6853,6 +6853,100 @@
         <v>RA-342/2026-SP-3</v>
       </c>
       <c s="2" t="str">
+        <v>Atendido</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Solicitamos o atendimento para fornecimento e utilização de água de REUSO na UTGC. Segue até a data, a informação para a devido fornecimento, onde permanece a penalização em DGI, até o efetivo e completo atendimento desta adequação.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em ateno ao RA-342/2026/SP-3, a CONTRATADA informa que a ETE da UTGC segue em operao regular, e a pendncia refere-se  adequao do sistema de distribuio de gua de reuso, j registrada no RA 660/2025 e ainda sem soluo definitiva.Propomos inspeo tcnica conjunta com a Fiscalizao para definio do escopo de adequao e do instrumento contratual aplicvel (OM, PPU ou alterao contratual).Solicitamos a suspenso do DGI at a concluso desse diagnstico conjunto.Permanecemos  disposio.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>30/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="137" ht="12.75">
+      <c r="A137" s="2" t="str">
+        <v>RA-357/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atendido</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Envio o levantamento de todos os pontos com ausência da sinalização de altura e das respectivas medidas, para que no prazo de até 15/08 parte destes pontos já estejam adequados.</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>A Normatel informa que o servio de Placas est em andamento comonde cerca de 36 Placas j foram instaladas, conforme relatrio em anexo. ,A instalao est alinhada com as solicitaes da Fiscalizao deste contrato e de acordo; com a programao do SAP.AtcEduardo WallaceGer. de ContratoNormatel Engenharia</v>
+      </c>
+      <c s="2" t="str">
+        <v>F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v>31/07/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Relatório de Placas de Altura e Ruas.pdf</v>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v>F1QM</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="138" ht="12.75">
+      <c r="A138" s="2" t="str">
+        <v>RA-368/2026-SP-4</v>
+      </c>
+      <c s="2" t="str">
         <v>Em Atendimento</v>
       </c>
       <c s="2" t="str">
@@ -6862,10 +6956,10 @@
         <v>UTGC</v>
       </c>
       <c s="2" t="str">
-        <v>Solicitamos o atendimento para fornecimento e utilização de água de REUSO na UTGC. Segue até a data, a informação para a devido fornecimento, onde permanece a penalização em DGI, até o efetivo e completo atendimento desta adequação.</v>
-      </c>
-      <c s="2" t="str">
-        <v>15/07/2026</v>
+        <v>Solicitamos que, após a conclusão das adequações, sejam encaminhadas as evidências das adequação.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/08/2026</v>
       </c>
       <c s="2" t="str">
         <v/>
@@ -6890,6 +6984,147 @@
       </c>
       <c s="2" t="str">
         <v/>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="139" ht="12.75">
+      <c r="A139" s="2" t="str">
+        <v>RA-380/2026-SP-3</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atendido</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Envio imediato dos laudos, bem como a apresentação de justificativa formal para o não atendimento e medidas de mitigação.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Foram realizadas as coletas nos pontos solicitados em 24/06/2026, conforme solicitado. Os laudos foram concludos em 03/07/2026.Seguem em anexo os laudos referentes s coletas realizadas.</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>206733-2026 - 1-0 k-55 portaria.pdf, 206739-2026 - 1-0 k-26 cozinha.pdf</v>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v>CIEA</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="140" ht="12.75">
+      <c r="A140" s="2" t="str">
+        <v>RA-382/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atendido</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>UTGC</v>
+      </c>
+      <c s="2" t="str">
+        <v>Enviar evidência de realização até a medição de Agosto/26.</v>
+      </c>
+      <c s="2" t="str">
+        <v>15/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>11/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>Prezados,Em atendimento  RA-382/2026, encaminhamos, em anexo, as evidncias dos treinamentos e dilogos ambientais realizados no perodo de fevereiro de 2026 at a presente data.A documentao apresentada contempla os materiais utilizados, as listas de presena e os registros fotogrficos das atividades realizadas, demonstrando as aes de conscientizao e capacitao ambiental que vm sendo desenvolvidas junto s equipes do contrato.Dessa forma, apresentamos as evidncias para avaliao da fiscalizao e solicitamos o encerramento da presente RA.Solange OliveiraNORMATEL ENGENHARIA</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v>11/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>1-DMMA - RESIDUO.jpeg, 260225- DMS - Gestão de residuos na UTGC.pdf, DMMA -02-06-2026.png, DMMA Abril - Pragas e Vetores.pdf, DMMA Maio -Dinamica de Residuos.pdf, DSMA - Agua -03-2026-05.jpeg, DSMS GERAL MÊS 07.pdf, DSMS MARÇO -26.pdf, DMMA -02-06-2026.png, DSMA - Agua -03-2026-05.jpeg</v>
+      </c>
+      <c s="2" t="str">
+        <v>MP00</v>
+      </c>
+      <c s="2" t="str">
+        <v>GK42</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141" ht="12.75">
+      <c r="A141" s="2" t="str">
+        <v>RA-387/2026-SP-1</v>
+      </c>
+      <c s="2" t="str">
+        <v>Atendido</v>
+      </c>
+      <c s="2" t="str">
+        <v>4600682358</v>
+      </c>
+      <c s="2" t="str">
+        <v>TIMS</v>
+      </c>
+      <c s="2" t="str">
+        <v>A fiscalização da Petrobras notifica a empresa Normatel pela falha no fechamento das Ordens de Manutenção 2032142295 e 2032142296 no sistema SAP impactando no ICPO. Solicita-se atenção para evitar a repetição desses eventos</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v>Registrado com Pendência</v>
+      </c>
+      <c s="2" t="str">
+        <v>A situao ocorreu devido a um erro de sincronizao no Sigabrizzo, sistema da Petrobras. As ordens foram encerradas manualmente pela equipe, porm houve um atraso na atualizao das informaes no sistema, o que acabou impactando o indicador do ICPO.</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
+      </c>
+      <c s="2" t="str">
+        <v>12/08/2026</v>
+      </c>
+      <c s="2" t="str">
+        <v/>
+      </c>
+      <c s="2" t="str">
+        <v>CMOL</v>
+      </c>
+      <c s="2" t="str">
+        <v>DUHJ</v>
       </c>
       <c s="2" t="str">
         <v/>

</xml_diff>